<commit_message>
5-26 merger the 2 vods together
</commit_message>
<xml_diff>
--- a/DorozeaStreamStats.xlsx
+++ b/DorozeaStreamStats.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="329">
   <si>
     <t>stream</t>
   </si>
@@ -995,6 +995,9 @@
   </si>
   <si>
     <t>jc, roblox, ftfN</t>
+  </si>
+  <si>
+    <t>jc, mc, 007</t>
   </si>
 </sst>
 </file>
@@ -12158,6 +12161,24 @@
         <v>10</v>
       </c>
     </row>
+    <row r="641">
+      <c r="A641" s="1">
+        <v>639.0</v>
+      </c>
+      <c r="B641" s="1">
+        <v>1285.0</v>
+      </c>
+      <c r="C641" s="1">
+        <v>1455.0</v>
+      </c>
+      <c r="D641" s="1">
+        <v>106.0</v>
+      </c>
+      <c r="E641" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F641" s="1"/>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>